<commit_message>
vault backup: 2026-04-24 17:44:18
</commit_message>
<xml_diff>
--- a/Knowledge/Model Schema/PG/Model Output/PG_model.xlsx
+++ b/Knowledge/Model Schema/PG/Model Output/PG_model.xlsx
@@ -18,8 +18,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="#,##0;(#,##0);&quot;--&quot;"/>
+    <numFmt numFmtId="165" formatCode="$#,##0_);($#,##0);&quot;$--&quot;_)"/>
   </numFmts>
   <fonts count="3">
     <font>
@@ -51,7 +52,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -59,11 +60,16 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <top style="thin">
+        <color rgb="00000000"/>
+      </top>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -71,6 +77,7 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -436,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -464,10 +471,10 @@
         </is>
       </c>
       <c r="B2" s="4" t="n">
-        <v>0</v>
+        <v>43619</v>
       </c>
       <c r="C2" s="4" t="n">
-        <v>21882</v>
+        <v>44594</v>
       </c>
     </row>
     <row r="3">
@@ -477,10 +484,10 @@
         </is>
       </c>
       <c r="B3" s="4" t="n">
-        <v>0</v>
+        <v>20839</v>
       </c>
       <c r="C3" s="4" t="n">
-        <v>10418</v>
+        <v>21721</v>
       </c>
     </row>
     <row r="4">
@@ -490,10 +497,10 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>0</v>
+        <v>11242</v>
       </c>
       <c r="C4" s="4" t="n">
-        <v>5723</v>
+        <v>11651</v>
       </c>
     </row>
     <row r="5">
@@ -503,10 +510,10 @@
         </is>
       </c>
       <c r="B5" s="4" t="n">
-        <v>0</v>
+        <v>11538</v>
       </c>
       <c r="C5" s="4" t="n">
-        <v>5741</v>
+        <v>11222</v>
       </c>
     </row>
     <row r="6">
@@ -516,10 +523,10 @@
         </is>
       </c>
       <c r="B6" s="4" t="n">
-        <v>0</v>
+        <v>-478</v>
       </c>
       <c r="C6" s="4" t="n">
-        <v>-240</v>
+        <v>-417</v>
       </c>
     </row>
     <row r="7">
@@ -529,10 +536,10 @@
         </is>
       </c>
       <c r="B7" s="4" t="n">
-        <v>0</v>
+        <v>254</v>
       </c>
       <c r="C7" s="4" t="n">
-        <v>119</v>
+        <v>222</v>
       </c>
     </row>
     <row r="8">
@@ -542,10 +549,10 @@
         </is>
       </c>
       <c r="B8" s="4" t="n">
-        <v>0</v>
+        <v>-330</v>
       </c>
       <c r="C8" s="4" t="n">
-        <v>224</v>
+        <v>427</v>
       </c>
     </row>
     <row r="9">
@@ -554,11 +561,13 @@
           <t>Pre-Tax Income (Loss)</t>
         </is>
       </c>
-      <c r="B9" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C9" s="4" t="n">
-        <v>5845</v>
+      <c r="B9" s="5">
+        <f>B5-SUM(B6:B8)</f>
+        <v/>
+      </c>
+      <c r="C9" s="5">
+        <f>C5-SUM(C6:C8)</f>
+        <v/>
       </c>
     </row>
     <row r="10">
@@ -568,10 +577,10 @@
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>0</v>
+        <v>-2339</v>
       </c>
       <c r="C10" s="4" t="n">
-        <v>-1187</v>
+        <v>-2343</v>
       </c>
     </row>
     <row r="11">
@@ -580,11 +589,13 @@
           <t>Net Income (Loss)</t>
         </is>
       </c>
-      <c r="B11" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C11" s="4" t="n">
-        <v>9289</v>
+      <c r="B11" s="5">
+        <f>B9-B10</f>
+        <v/>
+      </c>
+      <c r="C11" s="5">
+        <f>C9-C10</f>
+        <v/>
       </c>
     </row>
     <row r="12">
@@ -594,10 +605,10 @@
         </is>
       </c>
       <c r="B12" s="4" t="n">
-        <v>0</v>
+        <v>56</v>
       </c>
       <c r="C12" s="4" t="n">
-        <v>29</v>
+        <v>42</v>
       </c>
     </row>
     <row r="13">
@@ -607,10 +618,10 @@
         </is>
       </c>
       <c r="B13" s="4" t="n">
-        <v>0</v>
+        <v>3.59</v>
       </c>
       <c r="C13" s="4" t="n">
-        <v>1.94e-06</v>
+        <v>3.82</v>
       </c>
     </row>
     <row r="14">
@@ -620,23 +631,10 @@
         </is>
       </c>
       <c r="B14" s="4" t="n">
-        <v>0</v>
+        <v>3.49</v>
       </c>
       <c r="C14" s="4" t="n">
-        <v>1.88e-06</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>Depreciation &amp; Amortization</t>
-        </is>
-      </c>
-      <c r="B15" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C15" s="4" t="n">
-        <v>803</v>
+        <v>3.73</v>
       </c>
     </row>
   </sheetData>
@@ -650,7 +648,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:C28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -674,274 +672,364 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Cash &amp; Cash Equivalents</t>
+          <t>Accounts Receivable</t>
         </is>
       </c>
       <c r="B2" s="4" t="n">
-        <v>9556</v>
+        <v>6185</v>
       </c>
       <c r="C2" s="4" t="n">
-        <v>10825</v>
+        <v>6279</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Accounts Receivable</t>
+          <t>Prepaid Expenses</t>
         </is>
       </c>
       <c r="B3" s="4" t="n">
-        <v>6185</v>
+        <v>2100</v>
       </c>
       <c r="C3" s="4" t="n">
-        <v>6279</v>
+        <v>1666</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Prepaid Expenses</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="n">
-        <v>2100</v>
-      </c>
-      <c r="C4" s="4" t="n">
-        <v>1666</v>
+          <t>Total Current Assets</t>
+        </is>
+      </c>
+      <c r="B4" s="5">
+        <f>SUM(B2:B3)</f>
+        <v/>
+      </c>
+      <c r="C4" s="5">
+        <f>SUM(C2:C3)</f>
+        <v/>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Net PP&amp;E</t>
+          <t>Cash &amp; Cash Equivalents</t>
         </is>
       </c>
       <c r="B5" s="4" t="n">
-        <v>23897</v>
+        <v>9556</v>
       </c>
       <c r="C5" s="4" t="n">
-        <v>24487</v>
+        <v>10825</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Goodwill</t>
+          <t>Net PP&amp;E</t>
         </is>
       </c>
       <c r="B6" s="4" t="n">
-        <v>41650</v>
+        <v>23897</v>
       </c>
       <c r="C6" s="4" t="n">
-        <v>41665</v>
+        <v>24487</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Intangible Assets</t>
+          <t>Goodwill</t>
         </is>
       </c>
       <c r="B7" s="4" t="n">
-        <v>21910</v>
+        <v>41650</v>
       </c>
       <c r="C7" s="4" t="n">
-        <v>21737</v>
+        <v>41665</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Other Non-Current Assets</t>
+          <t>Intangible Assets</t>
         </is>
       </c>
       <c r="B8" s="4" t="n">
-        <v>12381</v>
+        <v>21910</v>
       </c>
       <c r="C8" s="4" t="n">
-        <v>12809</v>
+        <v>21737</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Accounts Payable</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="n">
-        <v>15227</v>
-      </c>
-      <c r="C9" s="4" t="n">
-        <v>15173</v>
+          <t>Total Assets</t>
+        </is>
+      </c>
+      <c r="B9" s="5">
+        <f>B4+SUM(B5:B8)</f>
+        <v/>
+      </c>
+      <c r="C9" s="5">
+        <f>C4+SUM(C5:C8)</f>
+        <v/>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Accrued Expenses</t>
+          <t>Accounts Payable</t>
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>11318</v>
+        <v>15227</v>
       </c>
       <c r="C10" s="4" t="n">
-        <v>10463</v>
+        <v>15173</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Current Portion of Long-Term Debt</t>
+          <t>Accrued Expenses</t>
         </is>
       </c>
       <c r="B11" s="4" t="n">
-        <v>9513</v>
+        <v>11318</v>
       </c>
       <c r="C11" s="4" t="n">
-        <v>11062</v>
+        <v>10463</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Long-Term Debt</t>
+          <t>Current Portion of Long-Term Debt</t>
         </is>
       </c>
       <c r="B12" s="4" t="n">
-        <v>24995</v>
+        <v>9513</v>
       </c>
       <c r="C12" s="4" t="n">
-        <v>25577</v>
+        <v>11062</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Deferred Tax Assets</t>
-        </is>
-      </c>
-      <c r="B13" s="4" t="n">
-        <v>5774</v>
-      </c>
-      <c r="C13" s="4" t="n">
-        <v>5974</v>
+          <t>Total Current Liabilities</t>
+        </is>
+      </c>
+      <c r="B13" s="5">
+        <f>SUM(B10:B12)</f>
+        <v/>
+      </c>
+      <c r="C13" s="5">
+        <f>SUM(C10:C12)</f>
+        <v/>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Other Non-Current Liabilities</t>
+          <t>Long-Term Debt</t>
         </is>
       </c>
       <c r="B14" s="4" t="n">
-        <v>6120</v>
+        <v>24995</v>
       </c>
       <c r="C14" s="4" t="n">
-        <v>5719</v>
+        <v>25577</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Convertible Preferred Stock</t>
+          <t>Other Non-Current Liabilities</t>
         </is>
       </c>
       <c r="B15" s="4" t="n">
-        <v>777</v>
+        <v>6120</v>
       </c>
       <c r="C15" s="4" t="n">
-        <v>767</v>
+        <v>5719</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>Common Stock</t>
-        </is>
-      </c>
-      <c r="B16" s="4" t="n">
-        <v>4009</v>
-      </c>
-      <c r="C16" s="4" t="n">
-        <v>4009</v>
+          <t>Total Liabilities</t>
+        </is>
+      </c>
+      <c r="B16" s="5">
+        <f>B13+SUM(B14:B15)</f>
+        <v/>
+      </c>
+      <c r="C16" s="5">
+        <f>C13+SUM(C14:C15)</f>
+        <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>Additional Paid-in Capital</t>
+          <t>Convertible Preferred Stock</t>
         </is>
       </c>
       <c r="B17" s="4" t="n">
-        <v>68770</v>
+        <v>777</v>
       </c>
       <c r="C17" s="4" t="n">
-        <v>69010</v>
+        <v>767</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>ESOP Debt Retirement Reserve</t>
+          <t>Common Stock</t>
         </is>
       </c>
       <c r="B18" s="4" t="n">
-        <v>-672</v>
+        <v>4009</v>
       </c>
       <c r="C18" s="4" t="n">
-        <v>-637</v>
+        <v>4009</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>Accumulated Other Comprehensive Income (Loss)</t>
+          <t>Additional Paid-in Capital</t>
         </is>
       </c>
       <c r="B19" s="4" t="n">
-        <v>-12143</v>
+        <v>68770</v>
       </c>
       <c r="C19" s="4" t="n">
-        <v>-12108</v>
+        <v>69010</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>Treasury Stock</t>
+          <t>ESOP Debt Retirement Reserve</t>
         </is>
       </c>
       <c r="B20" s="4" t="n">
-        <v>-138702</v>
+        <v>-672</v>
       </c>
       <c r="C20" s="4" t="n">
-        <v>-141981</v>
+        <v>-637</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>Retained Earnings (Accumulated Deficit)</t>
+          <t>Accumulated Other Comprehensive Income (Loss)</t>
         </is>
       </c>
       <c r="B21" s="4" t="n">
-        <v>129973</v>
+        <v>-12143</v>
       </c>
       <c r="C21" s="4" t="n">
-        <v>133981</v>
+        <v>-12108</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
+          <t>Treasury Stock</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="n">
+        <v>-138702</v>
+      </c>
+      <c r="C22" s="4" t="n">
+        <v>-141981</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>Retained Earnings (Accumulated Deficit)</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="n">
+        <v>129973</v>
+      </c>
+      <c r="C23" s="4" t="n">
+        <v>133981</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
           <t>Noncontrolling Interest</t>
         </is>
       </c>
-      <c r="B22" s="4" t="n">
+      <c r="B24" s="4" t="n">
         <v>272</v>
       </c>
-      <c r="C22" s="4" t="n">
+      <c r="C24" s="4" t="n">
         <v>276</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>Total Stockholders' Equity</t>
+        </is>
+      </c>
+      <c r="B25" s="5">
+        <f>SUM(B17:B24)</f>
+        <v/>
+      </c>
+      <c r="C25" s="5">
+        <f>SUM(C17:C24)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>Total Liabilities, Mezzanine &amp; Stockholders' Equity</t>
+        </is>
+      </c>
+      <c r="B26" s="5">
+        <f>B16+B25</f>
+        <v/>
+      </c>
+      <c r="C26" s="5">
+        <f>C16+C25</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>Other Non-Current Assets</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="n">
+        <v>12381</v>
+      </c>
+      <c r="C27" s="4" t="n">
+        <v>12809</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>Deferred Tax Assets</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="n">
+        <v>5774</v>
+      </c>
+      <c r="C28" s="4" t="n">
+        <v>5974</v>
       </c>
     </row>
   </sheetData>
@@ -955,7 +1043,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:C23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -967,13 +1055,299 @@
       <c r="A1" s="1" t="inlineStr"/>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>FY2025</t>
+          <t>Q2 FY2025</t>
         </is>
       </c>
       <c r="C1" s="2" t="inlineStr">
         <is>
-          <t>FY2026</t>
-        </is>
+          <t>Q2 FY2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Depreciation &amp; Amortization</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="n">
+        <v>1434</v>
+      </c>
+      <c r="C2" s="4" t="n">
+        <v>1563</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Stock-Based Compensation</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="n">
+        <v>241</v>
+      </c>
+      <c r="C3" s="4" t="n">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>(Benefit) Provision for Deferred Income Taxes</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="n">
+        <v>221</v>
+      </c>
+      <c r="C4" s="4" t="n">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Gain (Loss) on Disposal of PP&amp;E</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="n">
+        <v>-787</v>
+      </c>
+      <c r="C5" s="4" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Accounts Receivable</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="n">
+        <v>262</v>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Inventories</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="n">
+        <v>170</v>
+      </c>
+      <c r="C7" s="4" t="n">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Accounts Payable</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="n">
+        <v>-286</v>
+      </c>
+      <c r="C8" s="4" t="n">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Other Operating Items</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="n">
+        <v>1484</v>
+      </c>
+      <c r="C9" s="4" t="n">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Purchase of PP&amp;E</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="n">
+        <v>1918</v>
+      </c>
+      <c r="C10" s="4" t="n">
+        <v>2367</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Proceeds from Sale of Assets</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="n">
+        <v>47</v>
+      </c>
+      <c r="C11" s="4" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Acquisitions, Net of Cash Acquired</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="n">
+        <v>-6</v>
+      </c>
+      <c r="C12" s="4" t="n">
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Other Investing Activities</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="n">
+        <v>153</v>
+      </c>
+      <c r="C13" s="4" t="n">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Common Dividends</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="n">
+        <v>4886</v>
+      </c>
+      <c r="C14" s="4" t="n">
+        <v>5093</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Proceeds from Short-Term Debt</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="n">
+        <v>5905</v>
+      </c>
+      <c r="C15" s="4" t="n">
+        <v>4180</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Repayments of Short-Term Debt</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="n">
+        <v>-571</v>
+      </c>
+      <c r="C16" s="4" t="n">
+        <v>-3270</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Net Change in Other Short-Term Debt</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="n">
+        <v>-2705</v>
+      </c>
+      <c r="C17" s="4" t="n">
+        <v>-471</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>Proceeds from Issuance of Long-Term Debt</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="n">
+        <v>995</v>
+      </c>
+      <c r="C18" s="4" t="n">
+        <v>2652</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>Repayments of Long-Term Debt</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="n">
+        <v>-1478</v>
+      </c>
+      <c r="C19" s="4" t="n">
+        <v>-1005</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>Share Repurchases</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="n">
+        <v>4449</v>
+      </c>
+      <c r="C20" s="4" t="n">
+        <v>3528</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Stock Options &amp; Other Financing Activities</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="n">
+        <v>985</v>
+      </c>
+      <c r="C21" s="4" t="n">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>FX Effect on Cash</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="n">
+        <v>-144</v>
+      </c>
+      <c r="C22" s="4" t="n">
+        <v>-21</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>Net Change in Cash</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="n">
+        <v>748</v>
+      </c>
+      <c r="C23" s="4" t="n">
+        <v>1269</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
vault backup: 2026-04-24 17:49:30
</commit_message>
<xml_diff>
--- a/Knowledge/Model Schema/PG/Model Output/PG_model.xlsx
+++ b/Knowledge/Model Schema/PG/Model Output/PG_model.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -586,16 +586,14 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Net Income (Loss)</t>
-        </is>
-      </c>
-      <c r="B11" s="5">
-        <f>B9-B10</f>
-        <v/>
-      </c>
-      <c r="C11" s="5">
-        <f>C9-C10</f>
-        <v/>
+          <t>Net Income (Loss) Including NCI</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="n">
+        <v>8646</v>
+      </c>
+      <c r="C11" s="4" t="n">
+        <v>9112</v>
       </c>
     </row>
     <row r="12">
@@ -614,26 +612,41 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Basic Earnings (Loss) per Share</t>
-        </is>
-      </c>
-      <c r="B13" s="4" t="n">
-        <v>3.59</v>
-      </c>
-      <c r="C13" s="4" t="n">
-        <v>3.82</v>
+          <t>Net Income (Loss)</t>
+        </is>
+      </c>
+      <c r="B13" s="5">
+        <f>B9-SUM(B10:B12)</f>
+        <v/>
+      </c>
+      <c r="C13" s="5">
+        <f>C9-SUM(C10:C12)</f>
+        <v/>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
+          <t>Basic Earnings (Loss) per Share</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="n">
+        <v>3.59</v>
+      </c>
+      <c r="C14" s="4" t="n">
+        <v>3.82</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
           <t>Diluted Earnings (Loss) per Share</t>
         </is>
       </c>
-      <c r="B14" s="4" t="n">
+      <c r="B15" s="4" t="n">
         <v>3.49</v>
       </c>
-      <c r="C14" s="4" t="n">
+      <c r="C15" s="4" t="n">
         <v>3.73</v>
       </c>
     </row>
@@ -672,55 +685,55 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Accounts Receivable</t>
+          <t>Cash &amp; Cash Equivalents</t>
         </is>
       </c>
       <c r="B2" s="4" t="n">
-        <v>6185</v>
+        <v>9556</v>
       </c>
       <c r="C2" s="4" t="n">
-        <v>6279</v>
+        <v>10825</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Prepaid Expenses</t>
+          <t>Accounts Receivable</t>
         </is>
       </c>
       <c r="B3" s="4" t="n">
-        <v>2100</v>
+        <v>6185</v>
       </c>
       <c r="C3" s="4" t="n">
-        <v>1666</v>
+        <v>6279</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Total Current Assets</t>
-        </is>
-      </c>
-      <c r="B4" s="5">
-        <f>SUM(B2:B3)</f>
-        <v/>
-      </c>
-      <c r="C4" s="5">
-        <f>SUM(C2:C3)</f>
-        <v/>
+          <t>Prepaid Expenses</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="n">
+        <v>2100</v>
+      </c>
+      <c r="C4" s="4" t="n">
+        <v>1666</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Cash &amp; Cash Equivalents</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="n">
-        <v>9556</v>
-      </c>
-      <c r="C5" s="4" t="n">
-        <v>10825</v>
+          <t>Total Current Assets</t>
+        </is>
+      </c>
+      <c r="B5" s="5">
+        <f>SUM(B2:B4)</f>
+        <v/>
+      </c>
+      <c r="C5" s="5">
+        <f>SUM(C2:C4)</f>
+        <v/>
       </c>
     </row>
     <row r="6">
@@ -765,271 +778,271 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Total Assets</t>
-        </is>
-      </c>
-      <c r="B9" s="5">
-        <f>B4+SUM(B5:B8)</f>
-        <v/>
-      </c>
-      <c r="C9" s="5">
-        <f>C4+SUM(C5:C8)</f>
-        <v/>
+          <t>Other Non-Current Assets</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="n">
+        <v>12381</v>
+      </c>
+      <c r="C9" s="4" t="n">
+        <v>12809</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Accounts Payable</t>
+          <t>Deferred Tax Assets</t>
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>15227</v>
+        <v>5774</v>
       </c>
       <c r="C10" s="4" t="n">
-        <v>15173</v>
+        <v>5974</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Accrued Expenses</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="n">
-        <v>11318</v>
-      </c>
-      <c r="C11" s="4" t="n">
-        <v>10463</v>
+          <t>Total Assets</t>
+        </is>
+      </c>
+      <c r="B11" s="5">
+        <f>B5+SUM(B6:B10)</f>
+        <v/>
+      </c>
+      <c r="C11" s="5">
+        <f>C5+SUM(C6:C10)</f>
+        <v/>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Current Portion of Long-Term Debt</t>
+          <t>Accounts Payable</t>
         </is>
       </c>
       <c r="B12" s="4" t="n">
-        <v>9513</v>
+        <v>15227</v>
       </c>
       <c r="C12" s="4" t="n">
-        <v>11062</v>
+        <v>15173</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Total Current Liabilities</t>
-        </is>
-      </c>
-      <c r="B13" s="5">
-        <f>SUM(B10:B12)</f>
-        <v/>
-      </c>
-      <c r="C13" s="5">
-        <f>SUM(C10:C12)</f>
-        <v/>
+          <t>Accrued Expenses</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="n">
+        <v>11318</v>
+      </c>
+      <c r="C13" s="4" t="n">
+        <v>10463</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Long-Term Debt</t>
+          <t>Current Portion of Long-Term Debt</t>
         </is>
       </c>
       <c r="B14" s="4" t="n">
-        <v>24995</v>
+        <v>9513</v>
       </c>
       <c r="C14" s="4" t="n">
-        <v>25577</v>
+        <v>11062</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Other Non-Current Liabilities</t>
-        </is>
-      </c>
-      <c r="B15" s="4" t="n">
-        <v>6120</v>
-      </c>
-      <c r="C15" s="4" t="n">
-        <v>5719</v>
+          <t>Total Current Liabilities</t>
+        </is>
+      </c>
+      <c r="B15" s="5">
+        <f>SUM(B12:B14)</f>
+        <v/>
+      </c>
+      <c r="C15" s="5">
+        <f>SUM(C12:C14)</f>
+        <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>Total Liabilities</t>
-        </is>
-      </c>
-      <c r="B16" s="5">
-        <f>B13+SUM(B14:B15)</f>
-        <v/>
-      </c>
-      <c r="C16" s="5">
-        <f>C13+SUM(C14:C15)</f>
-        <v/>
+          <t>Long-Term Debt</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="n">
+        <v>24995</v>
+      </c>
+      <c r="C16" s="4" t="n">
+        <v>25577</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>Convertible Preferred Stock</t>
+          <t>Other Non-Current Liabilities</t>
         </is>
       </c>
       <c r="B17" s="4" t="n">
-        <v>777</v>
+        <v>6120</v>
       </c>
       <c r="C17" s="4" t="n">
-        <v>767</v>
+        <v>5719</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>Common Stock</t>
-        </is>
-      </c>
-      <c r="B18" s="4" t="n">
-        <v>4009</v>
-      </c>
-      <c r="C18" s="4" t="n">
-        <v>4009</v>
+          <t>Total Liabilities</t>
+        </is>
+      </c>
+      <c r="B18" s="5">
+        <f>B15+SUM(B16:B17)</f>
+        <v/>
+      </c>
+      <c r="C18" s="5">
+        <f>C15+SUM(C16:C17)</f>
+        <v/>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>Additional Paid-in Capital</t>
+          <t>Convertible Preferred Stock</t>
         </is>
       </c>
       <c r="B19" s="4" t="n">
-        <v>68770</v>
+        <v>777</v>
       </c>
       <c r="C19" s="4" t="n">
-        <v>69010</v>
+        <v>767</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>ESOP Debt Retirement Reserve</t>
+          <t>Common Stock</t>
         </is>
       </c>
       <c r="B20" s="4" t="n">
-        <v>-672</v>
+        <v>4009</v>
       </c>
       <c r="C20" s="4" t="n">
-        <v>-637</v>
+        <v>4009</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>Accumulated Other Comprehensive Income (Loss)</t>
+          <t>Additional Paid-in Capital</t>
         </is>
       </c>
       <c r="B21" s="4" t="n">
-        <v>-12143</v>
+        <v>68770</v>
       </c>
       <c r="C21" s="4" t="n">
-        <v>-12108</v>
+        <v>69010</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>Treasury Stock</t>
+          <t>ESOP Debt Retirement Reserve</t>
         </is>
       </c>
       <c r="B22" s="4" t="n">
-        <v>-138702</v>
+        <v>-672</v>
       </c>
       <c r="C22" s="4" t="n">
-        <v>-141981</v>
+        <v>-637</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>Retained Earnings (Accumulated Deficit)</t>
+          <t>Accumulated Other Comprehensive Income (Loss)</t>
         </is>
       </c>
       <c r="B23" s="4" t="n">
-        <v>129973</v>
+        <v>-12143</v>
       </c>
       <c r="C23" s="4" t="n">
-        <v>133981</v>
+        <v>-12108</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>Noncontrolling Interest</t>
+          <t>Treasury Stock</t>
         </is>
       </c>
       <c r="B24" s="4" t="n">
-        <v>272</v>
+        <v>-138702</v>
       </c>
       <c r="C24" s="4" t="n">
-        <v>276</v>
+        <v>-141981</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>Total Stockholders' Equity</t>
-        </is>
-      </c>
-      <c r="B25" s="5">
-        <f>SUM(B17:B24)</f>
-        <v/>
-      </c>
-      <c r="C25" s="5">
-        <f>SUM(C17:C24)</f>
-        <v/>
+          <t>Retained Earnings (Accumulated Deficit)</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="n">
+        <v>129973</v>
+      </c>
+      <c r="C25" s="4" t="n">
+        <v>133981</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>Total Liabilities, Mezzanine &amp; Stockholders' Equity</t>
-        </is>
-      </c>
-      <c r="B26" s="5">
-        <f>B16+B25</f>
-        <v/>
-      </c>
-      <c r="C26" s="5">
-        <f>C16+C25</f>
-        <v/>
+          <t>Noncontrolling Interest</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="n">
+        <v>272</v>
+      </c>
+      <c r="C26" s="4" t="n">
+        <v>276</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>Other Non-Current Assets</t>
-        </is>
-      </c>
-      <c r="B27" s="4" t="n">
-        <v>12381</v>
-      </c>
-      <c r="C27" s="4" t="n">
-        <v>12809</v>
+          <t>Total Stockholders' Equity</t>
+        </is>
+      </c>
+      <c r="B27" s="5">
+        <f>SUM(B19:B26)</f>
+        <v/>
+      </c>
+      <c r="C27" s="5">
+        <f>SUM(C19:C26)</f>
+        <v/>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>Deferred Tax Assets</t>
-        </is>
-      </c>
-      <c r="B28" s="4" t="n">
-        <v>5774</v>
-      </c>
-      <c r="C28" s="4" t="n">
-        <v>5974</v>
+          <t>Total Liabilities, Mezzanine &amp; Stockholders' Equity</t>
+        </is>
+      </c>
+      <c r="B28" s="5">
+        <f>B18+B27</f>
+        <v/>
+      </c>
+      <c r="C28" s="5">
+        <f>C18+C27</f>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
vault backup: 2026-04-25 14:13:22
</commit_message>
<xml_diff>
--- a/Knowledge/Model Schema/PG/Model Output/PG_model.xlsx
+++ b/Knowledge/Model Schema/PG/Model Output/PG_model.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -484,10 +484,10 @@
         </is>
       </c>
       <c r="B3" s="4" t="n">
-        <v>20839</v>
+        <v>-20839</v>
       </c>
       <c r="C3" s="4" t="n">
-        <v>21721</v>
+        <v>-21721</v>
       </c>
     </row>
     <row r="4">
@@ -497,10 +497,10 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>11242</v>
+        <v>-11242</v>
       </c>
       <c r="C4" s="4" t="n">
-        <v>11651</v>
+        <v>-11651</v>
       </c>
     </row>
     <row r="5">
@@ -519,134 +519,121 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Interest Expense</t>
+          <t>Interest Income (Expense)</t>
         </is>
       </c>
       <c r="B6" s="4" t="n">
-        <v>-478</v>
+        <v>732</v>
       </c>
       <c r="C6" s="4" t="n">
-        <v>-417</v>
+        <v>639</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Interest Income</t>
+          <t>Other Income (Expense)</t>
         </is>
       </c>
       <c r="B7" s="4" t="n">
-        <v>254</v>
+        <v>-330</v>
       </c>
       <c r="C7" s="4" t="n">
-        <v>222</v>
+        <v>427</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Other Income (Expense)</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="n">
-        <v>-330</v>
-      </c>
-      <c r="C8" s="4" t="n">
-        <v>427</v>
+          <t>Pre-Tax Income (Loss)</t>
+        </is>
+      </c>
+      <c r="B8" s="5">
+        <f>B5-SUM(B6:B7)</f>
+        <v/>
+      </c>
+      <c r="C8" s="5">
+        <f>C5-SUM(C6:C7)</f>
+        <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Pre-Tax Income (Loss)</t>
-        </is>
-      </c>
-      <c r="B9" s="5">
-        <f>B5-SUM(B6:B8)</f>
-        <v/>
-      </c>
-      <c r="C9" s="5">
-        <f>C5-SUM(C6:C8)</f>
-        <v/>
+          <t>Income Tax (Expense) Benefit</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="n">
+        <v>2339</v>
+      </c>
+      <c r="C9" s="4" t="n">
+        <v>2343</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Income Tax (Benefit) Expense</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="n">
-        <v>-2339</v>
-      </c>
-      <c r="C10" s="4" t="n">
-        <v>-2343</v>
+          <t>Net Income (Loss)</t>
+        </is>
+      </c>
+      <c r="B10" s="5">
+        <f>B8-B9</f>
+        <v/>
+      </c>
+      <c r="C10" s="5">
+        <f>C8-C9</f>
+        <v/>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Net Income (Loss) Including NCI</t>
+          <t>Net Income (Loss) Attributable to Noncontrolling Interest</t>
         </is>
       </c>
       <c r="B11" s="4" t="n">
-        <v>8646</v>
+        <v>56</v>
       </c>
       <c r="C11" s="4" t="n">
-        <v>9112</v>
+        <v>42</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Net Income (Loss) Attributable to Noncontrolling Interest</t>
+          <t>Net Income (Loss) Less NCI</t>
         </is>
       </c>
       <c r="B12" s="4" t="n">
-        <v>56</v>
+        <v>8589</v>
       </c>
       <c r="C12" s="4" t="n">
-        <v>42</v>
+        <v>9070</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Net Income (Loss)</t>
-        </is>
-      </c>
-      <c r="B13" s="5">
-        <f>B9-SUM(B10:B12)</f>
-        <v/>
-      </c>
-      <c r="C13" s="5">
-        <f>C9-SUM(C10:C12)</f>
-        <v/>
+          <t>Basic Earnings (Loss) per Share</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="n">
+        <v>3.59</v>
+      </c>
+      <c r="C13" s="4" t="n">
+        <v>3.82</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Basic Earnings (Loss) per Share</t>
+          <t>Diluted Earnings (Loss) per Share</t>
         </is>
       </c>
       <c r="B14" s="4" t="n">
-        <v>3.59</v>
+        <v>3.49</v>
       </c>
       <c r="C14" s="4" t="n">
-        <v>3.82</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>Diluted Earnings (Loss) per Share</t>
-        </is>
-      </c>
-      <c r="B15" s="4" t="n">
-        <v>3.49</v>
-      </c>
-      <c r="C15" s="4" t="n">
         <v>3.73</v>
       </c>
     </row>
@@ -661,7 +648,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C28"/>
+  <dimension ref="A1:C29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -711,94 +698,94 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Prepaid Expenses</t>
+          <t>Inventories</t>
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>2100</v>
+        <v>7551</v>
       </c>
       <c r="C4" s="4" t="n">
-        <v>1666</v>
+        <v>7817</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Total Current Assets</t>
-        </is>
-      </c>
-      <c r="B5" s="5">
-        <f>SUM(B2:B4)</f>
-        <v/>
-      </c>
-      <c r="C5" s="5">
-        <f>SUM(C2:C4)</f>
-        <v/>
+          <t>Prepaid Expenses</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="n">
+        <v>2100</v>
+      </c>
+      <c r="C5" s="4" t="n">
+        <v>1666</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Net PP&amp;E</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="n">
-        <v>23897</v>
-      </c>
-      <c r="C6" s="4" t="n">
-        <v>24487</v>
+          <t>Total Current Assets</t>
+        </is>
+      </c>
+      <c r="B6" s="5">
+        <f>SUM(B2:B5)</f>
+        <v/>
+      </c>
+      <c r="C6" s="5">
+        <f>SUM(C2:C5)</f>
+        <v/>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Goodwill</t>
+          <t>Net PP&amp;E</t>
         </is>
       </c>
       <c r="B7" s="4" t="n">
-        <v>41650</v>
+        <v>23897</v>
       </c>
       <c r="C7" s="4" t="n">
-        <v>41665</v>
+        <v>24487</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Intangible Assets</t>
+          <t>Goodwill</t>
         </is>
       </c>
       <c r="B8" s="4" t="n">
-        <v>21910</v>
+        <v>41650</v>
       </c>
       <c r="C8" s="4" t="n">
-        <v>21737</v>
+        <v>41665</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Other Non-Current Assets</t>
+          <t>Intangible Assets</t>
         </is>
       </c>
       <c r="B9" s="4" t="n">
-        <v>12381</v>
+        <v>21910</v>
       </c>
       <c r="C9" s="4" t="n">
-        <v>12809</v>
+        <v>21737</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Deferred Tax Assets</t>
+          <t>Other Non-Current Assets</t>
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>5774</v>
+        <v>12381</v>
       </c>
       <c r="C10" s="4" t="n">
-        <v>5974</v>
+        <v>12809</v>
       </c>
     </row>
     <row r="11">
@@ -808,11 +795,11 @@
         </is>
       </c>
       <c r="B11" s="5">
-        <f>B5+SUM(B6:B10)</f>
+        <f>B6+SUM(B7:B10)</f>
         <v/>
       </c>
       <c r="C11" s="5">
-        <f>C5+SUM(C6:C10)</f>
+        <f>C6+SUM(C7:C10)</f>
         <v/>
       </c>
     </row>
@@ -886,162 +873,175 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>Other Non-Current Liabilities</t>
+          <t>Deferred Tax Liability</t>
         </is>
       </c>
       <c r="B17" s="4" t="n">
-        <v>6120</v>
+        <v>5774</v>
       </c>
       <c r="C17" s="4" t="n">
-        <v>5719</v>
+        <v>5974</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>Total Liabilities</t>
-        </is>
-      </c>
-      <c r="B18" s="5">
-        <f>B15+SUM(B16:B17)</f>
-        <v/>
-      </c>
-      <c r="C18" s="5">
-        <f>C15+SUM(C16:C17)</f>
-        <v/>
+          <t>Other Non-Current Liabilities</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="n">
+        <v>6120</v>
+      </c>
+      <c r="C18" s="4" t="n">
+        <v>5719</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>Convertible Preferred Stock</t>
-        </is>
-      </c>
-      <c r="B19" s="4" t="n">
-        <v>777</v>
-      </c>
-      <c r="C19" s="4" t="n">
-        <v>767</v>
+          <t>Total Liabilities</t>
+        </is>
+      </c>
+      <c r="B19" s="5">
+        <f>B15+SUM(B16:B18)</f>
+        <v/>
+      </c>
+      <c r="C19" s="5">
+        <f>C15+SUM(C16:C18)</f>
+        <v/>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>Common Stock</t>
+          <t>Convertible Preferred Stock</t>
         </is>
       </c>
       <c r="B20" s="4" t="n">
-        <v>4009</v>
+        <v>777</v>
       </c>
       <c r="C20" s="4" t="n">
-        <v>4009</v>
+        <v>767</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>Additional Paid-in Capital</t>
+          <t>Common Stock</t>
         </is>
       </c>
       <c r="B21" s="4" t="n">
-        <v>68770</v>
+        <v>4009</v>
       </c>
       <c r="C21" s="4" t="n">
-        <v>69010</v>
+        <v>4009</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>ESOP Debt Retirement Reserve</t>
+          <t>Additional Paid-in Capital</t>
         </is>
       </c>
       <c r="B22" s="4" t="n">
-        <v>-672</v>
+        <v>68770</v>
       </c>
       <c r="C22" s="4" t="n">
-        <v>-637</v>
+        <v>69010</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>Accumulated Other Comprehensive Income (Loss)</t>
+          <t>ESOP Debt Retirement Reserve</t>
         </is>
       </c>
       <c r="B23" s="4" t="n">
-        <v>-12143</v>
+        <v>-672</v>
       </c>
       <c r="C23" s="4" t="n">
-        <v>-12108</v>
+        <v>-637</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>Treasury Stock</t>
+          <t>Accumulated Other Comprehensive Income (Loss)</t>
         </is>
       </c>
       <c r="B24" s="4" t="n">
-        <v>-138702</v>
+        <v>-12143</v>
       </c>
       <c r="C24" s="4" t="n">
-        <v>-141981</v>
+        <v>-12108</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>Retained Earnings (Accumulated Deficit)</t>
+          <t>Treasury Stock</t>
         </is>
       </c>
       <c r="B25" s="4" t="n">
-        <v>129973</v>
+        <v>-138702</v>
       </c>
       <c r="C25" s="4" t="n">
-        <v>133981</v>
+        <v>-141981</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>Noncontrolling Interest</t>
+          <t>Retained Earnings (Accumulated Deficit)</t>
         </is>
       </c>
       <c r="B26" s="4" t="n">
-        <v>272</v>
+        <v>129973</v>
       </c>
       <c r="C26" s="4" t="n">
-        <v>276</v>
+        <v>133981</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>Total Stockholders' Equity</t>
-        </is>
-      </c>
-      <c r="B27" s="5">
-        <f>SUM(B19:B26)</f>
-        <v/>
-      </c>
-      <c r="C27" s="5">
-        <f>SUM(C19:C26)</f>
-        <v/>
+          <t>Noncontrolling Interest</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="n">
+        <v>272</v>
+      </c>
+      <c r="C27" s="4" t="n">
+        <v>276</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
+          <t>Total Stockholders' Equity</t>
+        </is>
+      </c>
+      <c r="B28" s="5">
+        <f>SUM(B20:B27)</f>
+        <v/>
+      </c>
+      <c r="C28" s="5">
+        <f>SUM(C20:C27)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
           <t>Total Liabilities, Mezzanine &amp; Stockholders' Equity</t>
         </is>
       </c>
-      <c r="B28" s="5">
-        <f>B18+B27</f>
-        <v/>
-      </c>
-      <c r="C28" s="5">
-        <f>C18+C27</f>
+      <c r="B29" s="5">
+        <f>B19+B28</f>
+        <v/>
+      </c>
+      <c r="C29" s="5">
+        <f>C19+C28</f>
         <v/>
       </c>
     </row>
@@ -1056,7 +1056,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C23"/>
+  <dimension ref="A1:C27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -1080,286 +1080,344 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Depreciation &amp; Amortization</t>
+          <t>Net Income (Loss)</t>
         </is>
       </c>
       <c r="B2" s="4" t="n">
-        <v>1434</v>
+        <v>8646</v>
       </c>
       <c r="C2" s="4" t="n">
-        <v>1563</v>
+        <v>9112</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Stock-Based Compensation</t>
+          <t>Depreciation &amp; Amortization</t>
         </is>
       </c>
       <c r="B3" s="4" t="n">
-        <v>241</v>
+        <v>1434</v>
       </c>
       <c r="C3" s="4" t="n">
-        <v>262</v>
+        <v>1563</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>(Benefit) Provision for Deferred Income Taxes</t>
+          <t>Stock-Based Compensation</t>
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>221</v>
+        <v>241</v>
       </c>
       <c r="C4" s="4" t="n">
-        <v>196</v>
+        <v>262</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Gain (Loss) on Disposal of PP&amp;E</t>
+          <t>(Benefit) Provision for Deferred Income Taxes</t>
         </is>
       </c>
       <c r="B5" s="4" t="n">
-        <v>-787</v>
+        <v>221</v>
       </c>
       <c r="C5" s="4" t="n">
-        <v>-1</v>
+        <v>196</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Accounts Receivable</t>
+          <t>Gain (Loss) on Disposal of PP&amp;E</t>
         </is>
       </c>
       <c r="B6" s="4" t="n">
-        <v>262</v>
+        <v>-787</v>
       </c>
       <c r="C6" s="4" t="n">
-        <v>92</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Inventories</t>
+          <t>Accounts Receivable</t>
         </is>
       </c>
       <c r="B7" s="4" t="n">
-        <v>170</v>
+        <v>262</v>
       </c>
       <c r="C7" s="4" t="n">
-        <v>255</v>
+        <v>92</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Accounts Payable</t>
+          <t>Inventories</t>
         </is>
       </c>
       <c r="B8" s="4" t="n">
-        <v>-286</v>
+        <v>170</v>
       </c>
       <c r="C8" s="4" t="n">
-        <v>239</v>
+        <v>255</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Other Operating Items</t>
+          <t>Accounts Payable</t>
         </is>
       </c>
       <c r="B9" s="4" t="n">
-        <v>1484</v>
+        <v>-286</v>
       </c>
       <c r="C9" s="4" t="n">
-        <v>645</v>
+        <v>239</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Purchase of PP&amp;E</t>
+          <t>Other Operating Items</t>
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>1918</v>
+        <v>1484</v>
       </c>
       <c r="C10" s="4" t="n">
-        <v>2367</v>
+        <v>645</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Proceeds from Sale of Assets</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="n">
-        <v>47</v>
-      </c>
-      <c r="C11" s="4" t="n">
-        <v>16</v>
+          <t>Cash Flow from Operations</t>
+        </is>
+      </c>
+      <c r="B11" s="5">
+        <f>SUM(B2:B10)</f>
+        <v/>
+      </c>
+      <c r="C11" s="5">
+        <f>SUM(C2:C10)</f>
+        <v/>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Acquisitions, Net of Cash Acquired</t>
+          <t>Purchase of PP&amp;E</t>
         </is>
       </c>
       <c r="B12" s="4" t="n">
-        <v>-6</v>
+        <v>1918</v>
       </c>
       <c r="C12" s="4" t="n">
-        <v>-5</v>
+        <v>2367</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Other Investing Activities</t>
+          <t>Proceeds from Sale of Assets</t>
         </is>
       </c>
       <c r="B13" s="4" t="n">
-        <v>153</v>
+        <v>47</v>
       </c>
       <c r="C13" s="4" t="n">
-        <v>408</v>
+        <v>16</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Common Dividends</t>
+          <t>Acquisitions, Net of Cash Acquired</t>
         </is>
       </c>
       <c r="B14" s="4" t="n">
-        <v>4886</v>
+        <v>6</v>
       </c>
       <c r="C14" s="4" t="n">
-        <v>5093</v>
+        <v>5</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Proceeds from Short-Term Debt</t>
+          <t>Other Investing Activities</t>
         </is>
       </c>
       <c r="B15" s="4" t="n">
-        <v>5905</v>
+        <v>153</v>
       </c>
       <c r="C15" s="4" t="n">
-        <v>4180</v>
+        <v>408</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>Repayments of Short-Term Debt</t>
-        </is>
-      </c>
-      <c r="B16" s="4" t="n">
-        <v>-571</v>
-      </c>
-      <c r="C16" s="4" t="n">
-        <v>-3270</v>
+          <t>Cash Flow from Investing</t>
+        </is>
+      </c>
+      <c r="B16" s="5">
+        <f>SUM(B12:B15)</f>
+        <v/>
+      </c>
+      <c r="C16" s="5">
+        <f>SUM(C12:C15)</f>
+        <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>Net Change in Other Short-Term Debt</t>
+          <t>Common Dividends</t>
         </is>
       </c>
       <c r="B17" s="4" t="n">
-        <v>-2705</v>
+        <v>4886</v>
       </c>
       <c r="C17" s="4" t="n">
-        <v>-471</v>
+        <v>5093</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>Proceeds from Issuance of Long-Term Debt</t>
+          <t>Proceeds from Short-Term Debt</t>
         </is>
       </c>
       <c r="B18" s="4" t="n">
-        <v>995</v>
+        <v>5905</v>
       </c>
       <c r="C18" s="4" t="n">
-        <v>2652</v>
+        <v>4180</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>Repayments of Long-Term Debt</t>
+          <t>Repayments of Short-Term Debt</t>
         </is>
       </c>
       <c r="B19" s="4" t="n">
-        <v>-1478</v>
+        <v>571</v>
       </c>
       <c r="C19" s="4" t="n">
-        <v>-1005</v>
+        <v>3270</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>Share Repurchases</t>
+          <t>Net Change in Other Short-Term Debt</t>
         </is>
       </c>
       <c r="B20" s="4" t="n">
-        <v>4449</v>
+        <v>-2705</v>
       </c>
       <c r="C20" s="4" t="n">
-        <v>3528</v>
+        <v>-471</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>Stock Options &amp; Other Financing Activities</t>
+          <t>Proceeds from Issuance of Long-Term Debt</t>
         </is>
       </c>
       <c r="B21" s="4" t="n">
-        <v>985</v>
+        <v>995</v>
       </c>
       <c r="C21" s="4" t="n">
-        <v>208</v>
+        <v>2652</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>FX Effect on Cash</t>
+          <t>Repayments of Long-Term Debt</t>
         </is>
       </c>
       <c r="B22" s="4" t="n">
-        <v>-144</v>
+        <v>1478</v>
       </c>
       <c r="C22" s="4" t="n">
-        <v>-21</v>
+        <v>1005</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
+          <t>Share Repurchases</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="n">
+        <v>4449</v>
+      </c>
+      <c r="C23" s="4" t="n">
+        <v>3528</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>Stock Options &amp; Other Financing Activities</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="n">
+        <v>985</v>
+      </c>
+      <c r="C24" s="4" t="n">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>Cash Flow from Financing</t>
+        </is>
+      </c>
+      <c r="B25" s="5">
+        <f>SUM(B17:B24)</f>
+        <v/>
+      </c>
+      <c r="C25" s="5">
+        <f>SUM(C17:C24)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>FX Effect on Cash</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="n">
+        <v>-144</v>
+      </c>
+      <c r="C26" s="4" t="n">
+        <v>-21</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
           <t>Net Change in Cash</t>
         </is>
       </c>
-      <c r="B23" s="4" t="n">
+      <c r="B27" s="4" t="n">
         <v>748</v>
       </c>
-      <c r="C23" s="4" t="n">
+      <c r="C27" s="4" t="n">
         <v>1269</v>
       </c>
     </row>

</xml_diff>